<commit_message>
Update BarrelIQ live data
</commit_message>
<xml_diff>
--- a/outputs/daily/hr_rankings_2026-06-16.xlsx
+++ b/outputs/daily/hr_rankings_2026-06-16.xlsx
@@ -65319,27 +65319,27 @@
       </c>
       <c r="B236" t="inlineStr">
         <is>
-          <t>676609</t>
+          <t>669242</t>
         </is>
       </c>
       <c r="C236" t="inlineStr">
         <is>
-          <t>Jose Caballero</t>
+          <t>Tommy Edman</t>
         </is>
       </c>
       <c r="D236" t="inlineStr">
         <is>
-          <t>NYY</t>
+          <t>LAD</t>
         </is>
       </c>
       <c r="E236" t="inlineStr">
         <is>
-          <t>CWS</t>
+          <t>TB</t>
         </is>
       </c>
       <c r="F236" t="inlineStr">
         <is>
-          <t>2026-06-16T23:05:00Z</t>
+          <t>2026-06-17T02:10:00Z</t>
         </is>
       </c>
       <c r="G236" t="inlineStr">
@@ -65349,17 +65349,17 @@
       </c>
       <c r="H236" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>9</t>
         </is>
       </c>
       <c r="I236" t="inlineStr">
         <is>
-          <t>Davis Martin</t>
+          <t>Drew Rasmussen</t>
         </is>
       </c>
       <c r="J236" t="inlineStr">
         <is>
-          <t>663436</t>
+          <t>656876</t>
         </is>
       </c>
       <c r="K236" t="inlineStr">
@@ -65368,7 +65368,7 @@
         </is>
       </c>
       <c r="L236" t="n">
-        <v>32.9</v>
+        <v>33.1</v>
       </c>
       <c r="M236" t="inlineStr">
         <is>
@@ -65382,27 +65382,27 @@
       </c>
       <c r="O236" t="inlineStr">
         <is>
-          <t>Projected Lineup</t>
+          <t>Projected Lineup, Platoon Edge</t>
         </is>
       </c>
       <c r="P236" t="n">
-        <v>8</v>
+        <v>24.6</v>
       </c>
       <c r="Q236" t="n">
-        <v>40.6</v>
+        <v>24.8</v>
       </c>
       <c r="R236" t="n">
-        <v>38.2</v>
+        <v>27.6</v>
       </c>
       <c r="S236" t="n">
-        <v>59.8</v>
+        <v>40.2</v>
       </c>
       <c r="T236" t="n">
+        <v>75</v>
+      </c>
+      <c r="U236" t="n">
         <v>50</v>
       </c>
-      <c r="U236" t="n">
-        <v>37.8</v>
-      </c>
       <c r="V236" t="inlineStr">
         <is>
           <t>No</t>
@@ -65415,7 +65415,7 @@
       </c>
       <c r="X236" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>9</t>
         </is>
       </c>
       <c r="Y236" t="inlineStr">
@@ -65440,7 +65440,7 @@
       </c>
       <c r="AC236" t="inlineStr">
         <is>
-          <t>H:2026/2025 P:2026/2025</t>
+          <t>H:2025 P:2026/2025</t>
         </is>
       </c>
       <c r="AD236" t="inlineStr"/>
@@ -65452,32 +65452,32 @@
       </c>
       <c r="AG236" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AH236" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AI236" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AJ236" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AK236" t="inlineStr">
         <is>
-          <t>Last 7 games: 6/24, 1 HR</t>
+          <t>Recent form unavailable</t>
         </is>
       </c>
       <c r="AL236" t="inlineStr">
         <is>
-          <t>same-side matchup; pitcher baseline 7.3% barrel, 8.1 HR allowed</t>
+          <t>switch hitter; pitcher baseline 6.7% barrel, 11.0 HR allowed</t>
         </is>
       </c>
       <c r="AM236" t="inlineStr">
@@ -65487,104 +65487,104 @@
       </c>
       <c r="AN236" t="inlineStr">
         <is>
-          <t>4.08</t>
+          <t>4.5</t>
         </is>
       </c>
       <c r="AO236" t="inlineStr">
         <is>
-          <t>27.94</t>
+          <t>39.9</t>
         </is>
       </c>
       <c r="AP236" t="inlineStr">
         <is>
-          <t>84.18</t>
+          <t>88.3</t>
         </is>
       </c>
       <c r="AQ236" t="inlineStr">
         <is>
-          <t>96.6061</t>
+          <t>99.3681</t>
         </is>
       </c>
       <c r="AR236" t="inlineStr">
         <is>
-          <t>0.3404</t>
+          <t>0.411</t>
         </is>
       </c>
       <c r="AS236" t="inlineStr">
         <is>
-          <t>0.1087</t>
+          <t>0.137</t>
         </is>
       </c>
       <c r="AT236" t="inlineStr">
         <is>
-          <t>0.2892</t>
+          <t>0.321</t>
         </is>
       </c>
       <c r="AU236" t="inlineStr">
         <is>
-          <t>68.82</t>
+          <t>70.2</t>
         </is>
       </c>
       <c r="AV236" t="inlineStr">
         <is>
-          <t>7.03</t>
+          <t>12.0</t>
         </is>
       </c>
       <c r="AW236" t="inlineStr">
         <is>
-          <t>39.15</t>
+          <t>42.6</t>
         </is>
       </c>
       <c r="AX236" t="inlineStr">
         <is>
-          <t>19.98</t>
+          <t>24.4</t>
         </is>
       </c>
       <c r="AY236" t="inlineStr">
         <is>
-          <t>5.7</t>
+          <t>13.0</t>
         </is>
       </c>
       <c r="AZ236" t="inlineStr">
         <is>
-          <t>0.1341</t>
+          <t>0.157</t>
         </is>
       </c>
       <c r="BA236" t="inlineStr">
         <is>
-          <t>7.28</t>
+          <t>6.65</t>
         </is>
       </c>
       <c r="BB236" t="inlineStr">
         <is>
-          <t>45.93</t>
+          <t>35.11</t>
         </is>
       </c>
       <c r="BC236" t="inlineStr">
         <is>
-          <t>90.35</t>
+          <t>87.8</t>
         </is>
       </c>
       <c r="BD236" t="inlineStr">
         <is>
-          <t>0.4097</t>
+          <t>0.3533</t>
         </is>
       </c>
       <c r="BE236" t="inlineStr">
         <is>
-          <t>0.1454</t>
+          <t>0.1229</t>
         </is>
       </c>
       <c r="BF236" t="inlineStr">
         <is>
-          <t>21.45</t>
+          <t>20.93</t>
         </is>
       </c>
       <c r="BG236" t="inlineStr"/>
       <c r="BH236" t="inlineStr"/>
       <c r="BI236" t="inlineStr">
         <is>
-          <t>Yankee Stadium</t>
+          <t>UNIQLO Field at Dodger Stadium</t>
         </is>
       </c>
       <c r="BJ236" t="inlineStr"/>
@@ -65595,27 +65595,27 @@
       </c>
       <c r="B237" t="inlineStr">
         <is>
-          <t>677587</t>
+          <t>676609</t>
         </is>
       </c>
       <c r="C237" t="inlineStr">
         <is>
-          <t>Brayan Rocchio</t>
+          <t>Jose Caballero</t>
         </is>
       </c>
       <c r="D237" t="inlineStr">
         <is>
-          <t>CLE</t>
+          <t>NYY</t>
         </is>
       </c>
       <c r="E237" t="inlineStr">
         <is>
-          <t>MIL</t>
+          <t>CWS</t>
         </is>
       </c>
       <c r="F237" t="inlineStr">
         <is>
-          <t>2026-06-16T23:40:00Z</t>
+          <t>2026-06-16T23:05:00Z</t>
         </is>
       </c>
       <c r="G237" t="inlineStr">
@@ -65625,26 +65625,26 @@
       </c>
       <c r="H237" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>7</t>
         </is>
       </c>
       <c r="I237" t="inlineStr">
         <is>
-          <t>Robert Gasser</t>
+          <t>Davis Martin</t>
         </is>
       </c>
       <c r="J237" t="inlineStr">
         <is>
-          <t>688107</t>
+          <t>663436</t>
         </is>
       </c>
       <c r="K237" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>R</t>
         </is>
       </c>
       <c r="L237" t="n">
-        <v>32.4</v>
+        <v>32.9</v>
       </c>
       <c r="M237" t="inlineStr">
         <is>
@@ -65658,26 +65658,26 @@
       </c>
       <c r="O237" t="inlineStr">
         <is>
-          <t>Projected Lineup, Platoon Edge</t>
+          <t>Projected Lineup</t>
         </is>
       </c>
       <c r="P237" t="n">
-        <v>14.8</v>
+        <v>8</v>
       </c>
       <c r="Q237" t="n">
-        <v>38.7</v>
+        <v>40.6</v>
       </c>
       <c r="R237" t="n">
-        <v>27.6</v>
+        <v>38.2</v>
       </c>
       <c r="S237" t="n">
-        <v>40.2</v>
+        <v>59.8</v>
       </c>
       <c r="T237" t="n">
-        <v>75</v>
+        <v>50</v>
       </c>
       <c r="U237" t="n">
-        <v>34.4</v>
+        <v>37.8</v>
       </c>
       <c r="V237" t="inlineStr">
         <is>
@@ -65691,7 +65691,7 @@
       </c>
       <c r="X237" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>7</t>
         </is>
       </c>
       <c r="Y237" t="inlineStr">
@@ -65733,12 +65733,12 @@
       </c>
       <c r="AH237" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="AI237" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>24</t>
         </is>
       </c>
       <c r="AJ237" t="inlineStr">
@@ -65748,119 +65748,119 @@
       </c>
       <c r="AK237" t="inlineStr">
         <is>
-          <t>Last 7 games: 5/22, 1 HR</t>
+          <t>Last 7 games: 6/24, 1 HR</t>
         </is>
       </c>
       <c r="AL237" t="inlineStr">
         <is>
-          <t>switch hitter; pitcher baseline 9.6% barrel, 4.5 HR allowed</t>
+          <t>same-side matchup; pitcher baseline 7.3% barrel, 8.1 HR allowed</t>
         </is>
       </c>
       <c r="AM237" t="inlineStr">
         <is>
-          <t>neutral batted-ball profile; pitcher allows elevated contact</t>
+          <t>neutral batted-ball profile; pitcher fly-ball pressure modest</t>
         </is>
       </c>
       <c r="AN237" t="inlineStr">
         <is>
-          <t>3.16</t>
+          <t>4.08</t>
         </is>
       </c>
       <c r="AO237" t="inlineStr">
         <is>
-          <t>33.89</t>
+          <t>27.94</t>
         </is>
       </c>
       <c r="AP237" t="inlineStr">
         <is>
-          <t>87.16</t>
+          <t>84.18</t>
         </is>
       </c>
       <c r="AQ237" t="inlineStr">
         <is>
-          <t>97.8268</t>
+          <t>96.6061</t>
         </is>
       </c>
       <c r="AR237" t="inlineStr">
         <is>
-          <t>0.3629</t>
+          <t>0.3404</t>
         </is>
       </c>
       <c r="AS237" t="inlineStr">
         <is>
-          <t>0.1102</t>
+          <t>0.1087</t>
         </is>
       </c>
       <c r="AT237" t="inlineStr">
         <is>
-          <t>0.3104</t>
+          <t>0.2892</t>
         </is>
       </c>
       <c r="AU237" t="inlineStr">
         <is>
-          <t>70.0</t>
+          <t>68.82</t>
         </is>
       </c>
       <c r="AV237" t="inlineStr">
         <is>
-          <t>7.29</t>
+          <t>7.03</t>
         </is>
       </c>
       <c r="AW237" t="inlineStr">
         <is>
-          <t>43.29</t>
+          <t>39.15</t>
         </is>
       </c>
       <c r="AX237" t="inlineStr">
         <is>
-          <t>22.43</t>
+          <t>19.98</t>
         </is>
       </c>
       <c r="AY237" t="inlineStr">
         <is>
-          <t>5.0</t>
+          <t>5.7</t>
         </is>
       </c>
       <c r="AZ237" t="inlineStr">
         <is>
-          <t>0.1196</t>
+          <t>0.1341</t>
         </is>
       </c>
       <c r="BA237" t="inlineStr">
         <is>
-          <t>9.56</t>
+          <t>7.28</t>
         </is>
       </c>
       <c r="BB237" t="inlineStr">
         <is>
-          <t>34.6</t>
+          <t>45.93</t>
         </is>
       </c>
       <c r="BC237" t="inlineStr">
         <is>
-          <t>88.41</t>
+          <t>90.35</t>
         </is>
       </c>
       <c r="BD237" t="inlineStr">
         <is>
-          <t>0.3701</t>
+          <t>0.4097</t>
         </is>
       </c>
       <c r="BE237" t="inlineStr">
         <is>
-          <t>0.1726</t>
+          <t>0.1454</t>
         </is>
       </c>
       <c r="BF237" t="inlineStr">
         <is>
-          <t>30.39</t>
+          <t>21.45</t>
         </is>
       </c>
       <c r="BG237" t="inlineStr"/>
       <c r="BH237" t="inlineStr"/>
       <c r="BI237" t="inlineStr">
         <is>
-          <t>American Family Field</t>
+          <t>Yankee Stadium</t>
         </is>
       </c>
       <c r="BJ237" t="inlineStr"/>
@@ -65871,27 +65871,27 @@
       </c>
       <c r="B238" t="inlineStr">
         <is>
-          <t>690976</t>
+          <t>677587</t>
         </is>
       </c>
       <c r="C238" t="inlineStr">
         <is>
-          <t>Alex Freeland</t>
+          <t>Brayan Rocchio</t>
         </is>
       </c>
       <c r="D238" t="inlineStr">
         <is>
-          <t>LAD</t>
+          <t>CLE</t>
         </is>
       </c>
       <c r="E238" t="inlineStr">
         <is>
-          <t>TB</t>
+          <t>MIL</t>
         </is>
       </c>
       <c r="F238" t="inlineStr">
         <is>
-          <t>2026-06-17T02:10:00Z</t>
+          <t>2026-06-16T23:40:00Z</t>
         </is>
       </c>
       <c r="G238" t="inlineStr">
@@ -65906,17 +65906,17 @@
       </c>
       <c r="I238" t="inlineStr">
         <is>
-          <t>Drew Rasmussen</t>
+          <t>Robert Gasser</t>
         </is>
       </c>
       <c r="J238" t="inlineStr">
         <is>
-          <t>656876</t>
+          <t>688107</t>
         </is>
       </c>
       <c r="K238" t="inlineStr">
         <is>
-          <t>R</t>
+          <t>L</t>
         </is>
       </c>
       <c r="L238" t="n">
@@ -65938,10 +65938,10 @@
         </is>
       </c>
       <c r="P238" t="n">
-        <v>28.6</v>
+        <v>14.8</v>
       </c>
       <c r="Q238" t="n">
-        <v>24.8</v>
+        <v>38.7</v>
       </c>
       <c r="R238" t="n">
         <v>27.6</v>
@@ -65953,7 +65953,7 @@
         <v>75</v>
       </c>
       <c r="U238" t="n">
-        <v>10.1</v>
+        <v>34.4</v>
       </c>
       <c r="V238" t="inlineStr">
         <is>
@@ -66009,134 +66009,134 @@
       </c>
       <c r="AH238" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>5</t>
         </is>
       </c>
       <c r="AI238" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>22</t>
         </is>
       </c>
       <c r="AJ238" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="AK238" t="inlineStr">
         <is>
-          <t>Last 7 games: 3/16, 0 HR</t>
+          <t>Last 7 games: 5/22, 1 HR</t>
         </is>
       </c>
       <c r="AL238" t="inlineStr">
         <is>
-          <t>switch hitter; pitcher baseline 6.7% barrel, 11.0 HR allowed</t>
+          <t>switch hitter; pitcher baseline 9.6% barrel, 4.5 HR allowed</t>
         </is>
       </c>
       <c r="AM238" t="inlineStr">
         <is>
-          <t>neutral batted-ball profile; pitcher fly-ball pressure modest</t>
+          <t>neutral batted-ball profile; pitcher allows elevated contact</t>
         </is>
       </c>
       <c r="AN238" t="inlineStr">
         <is>
-          <t>7.3</t>
+          <t>3.16</t>
         </is>
       </c>
       <c r="AO238" t="inlineStr">
         <is>
-          <t>39.4</t>
+          <t>33.89</t>
         </is>
       </c>
       <c r="AP238" t="inlineStr">
         <is>
-          <t>89.93</t>
+          <t>87.16</t>
         </is>
       </c>
       <c r="AQ238" t="inlineStr">
         <is>
-          <t>99.095</t>
+          <t>97.8268</t>
         </is>
       </c>
       <c r="AR238" t="inlineStr">
         <is>
-          <t>0.3319</t>
+          <t>0.3629</t>
         </is>
       </c>
       <c r="AS238" t="inlineStr">
         <is>
-          <t>0.1273</t>
+          <t>0.1102</t>
         </is>
       </c>
       <c r="AT238" t="inlineStr">
         <is>
-          <t>0.2838</t>
+          <t>0.3104</t>
         </is>
       </c>
       <c r="AU238" t="inlineStr">
         <is>
-          <t>70.7</t>
+          <t>70.0</t>
         </is>
       </c>
       <c r="AV238" t="inlineStr">
         <is>
-          <t>10.03</t>
+          <t>7.29</t>
         </is>
       </c>
       <c r="AW238" t="inlineStr">
         <is>
-          <t>34.5</t>
+          <t>43.29</t>
         </is>
       </c>
       <c r="AX238" t="inlineStr">
         <is>
-          <t>28.0</t>
+          <t>22.43</t>
         </is>
       </c>
       <c r="AY238" t="inlineStr">
         <is>
-          <t>2.7</t>
+          <t>5.0</t>
         </is>
       </c>
       <c r="AZ238" t="inlineStr">
         <is>
-          <t>0.1116</t>
+          <t>0.1196</t>
         </is>
       </c>
       <c r="BA238" t="inlineStr">
         <is>
-          <t>6.65</t>
+          <t>9.56</t>
         </is>
       </c>
       <c r="BB238" t="inlineStr">
         <is>
-          <t>35.11</t>
+          <t>34.6</t>
         </is>
       </c>
       <c r="BC238" t="inlineStr">
         <is>
-          <t>87.8</t>
+          <t>88.41</t>
         </is>
       </c>
       <c r="BD238" t="inlineStr">
         <is>
-          <t>0.3533</t>
+          <t>0.3701</t>
         </is>
       </c>
       <c r="BE238" t="inlineStr">
         <is>
-          <t>0.1229</t>
+          <t>0.1726</t>
         </is>
       </c>
       <c r="BF238" t="inlineStr">
         <is>
-          <t>20.93</t>
+          <t>30.39</t>
         </is>
       </c>
       <c r="BG238" t="inlineStr"/>
       <c r="BH238" t="inlineStr"/>
       <c r="BI238" t="inlineStr">
         <is>
-          <t>UNIQLO Field at Dodger Stadium</t>
+          <t>American Family Field</t>
         </is>
       </c>
       <c r="BJ238" t="inlineStr"/>

</xml_diff>